<commit_message>
Test Suite name modification
</commit_message>
<xml_diff>
--- a/KatalonData/ABPTestDataDemo/SchedulePaymentABP_NoCF_Demo.xlsx
+++ b/KatalonData/ABPTestDataDemo/SchedulePaymentABP_NoCF_Demo.xlsx
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="48">
   <si>
     <t>Result</t>
   </si>
@@ -265,6 +265,9 @@
   </si>
   <si>
     <t>Mon Jul 06 15:24:38 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jul 21 19:12:53 IST 2026</t>
   </si>
 </sst>
 </file>
@@ -1140,7 +1143,7 @@
         <v>14</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C2" s="4"/>
       <c r="D2" s="5" t="s">

</xml_diff>